<commit_message>
feat(lgo): catalogues TOP 200/300/500 au format exact de chaque logiciel, prix nets réels
Colonnes, ordre, ligne de titre, encodage et décimales alignés sur l'outil
catalogue d'Intégral (Winpharma 29 colonnes, Smart RX 15, Pharmaland 10,
Pharmony 4, LGPI 3) ; code article, TVA et prix net PC60 lus dans les fichiers
du 28/09. Le classement reste le nôtre : nombre de pharmacies du réseau.
Modes d'emploi et pas-à-pas mis en accord. Jeton 20261001lgo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/crm/v2/lgo/integral-top200-leo.xlsx
+++ b/crm/v2/lgo/integral-top200-leo.xlsx
@@ -533,7 +533,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>3474419</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>3400934744198</t>
@@ -571,7 +575,11 @@
       <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>4960553</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>3400949605538</t>
@@ -609,7 +617,11 @@
       <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>3200509</t>
+        </is>
+      </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>3400932005093</t>
@@ -647,7 +659,11 @@
       <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>6223413</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -685,7 +701,11 @@
       <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>3324737</t>
+        </is>
+      </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>3400933247379</t>
@@ -723,7 +743,11 @@
       <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>3515495</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>3400935154958</t>
@@ -761,7 +785,11 @@
       <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>3098608</t>
+        </is>
+      </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
           <t>3400930986080</t>
@@ -799,7 +827,11 @@
       <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>3029291</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>3400930292914</t>
@@ -815,7 +847,7 @@
         <v>221.32</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>212.71</v>
+        <v>212.74</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -837,7 +869,11 @@
       <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2238562</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
           <t>3400922385624</t>
@@ -875,7 +911,11 @@
       <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>3290599</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
           <t>3400932905997</t>
@@ -913,7 +953,11 @@
       <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>3029290</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>3400930292907</t>
@@ -929,7 +973,7 @@
         <v>163.7</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>157.33</v>
+        <v>157.36</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -951,7 +995,11 @@
       <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3443873</t>
+        </is>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>3400934438738</t>
@@ -989,7 +1037,11 @@
       <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>6042767</t>
+        </is>
+      </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -1027,7 +1079,11 @@
       <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>4066958</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1121,11 @@
       <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>3216290</t>
+        </is>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t>3400932162901</t>
@@ -1103,7 +1163,11 @@
       <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>3005620</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
           <t>3400930056202</t>
@@ -1119,7 +1183,7 @@
         <v>107.56</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>103.38</v>
+        <v>103.4</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -1141,7 +1205,11 @@
       <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>3138414</t>
+        </is>
+      </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
           <t>3400931384144</t>
@@ -1179,7 +1247,11 @@
       <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>3130737</t>
+        </is>
+      </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
           <t>3400931307372</t>
@@ -1217,7 +1289,11 @@
       <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>3552898</t>
+        </is>
+      </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
           <t>3400935528988</t>
@@ -1255,7 +1331,11 @@
       <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2686303</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
           <t>3400926863036</t>
@@ -1271,7 +1351,7 @@
         <v>73.34</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>70.48999999999999</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -1293,7 +1373,11 @@
       <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>3267672</t>
+        </is>
+      </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
           <t>3400932676729</t>
@@ -1331,7 +1415,11 @@
       <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>3034844</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
           <t>3400930348444</t>
@@ -1369,7 +1457,11 @@
       <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>3186301</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
           <t>3400931863014</t>
@@ -1407,7 +1499,11 @@
       <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>3019275</t>
+        </is>
+      </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
           <t>3400930192757</t>
@@ -1445,7 +1541,11 @@
       <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>3309525</t>
+        </is>
+      </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
           <t>3400933095253</t>
@@ -1483,7 +1583,11 @@
       <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>3171050</t>
+        </is>
+      </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
           <t>3400931710509</t>
@@ -1521,7 +1625,11 @@
       <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>3535836</t>
+        </is>
+      </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
           <t>3400935358363</t>
@@ -1559,7 +1667,11 @@
       <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>3479670</t>
+        </is>
+      </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
           <t>3400934796708</t>
@@ -1597,7 +1709,11 @@
       <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>3234017</t>
+        </is>
+      </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
           <t>3400932340170</t>
@@ -1635,7 +1751,11 @@
       <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>3014186</t>
+        </is>
+      </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
           <t>3400930141861</t>
@@ -1651,7 +1771,7 @@
         <v>175.18</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>168.37</v>
+        <v>168.39</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -1673,7 +1793,11 @@
       <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>3006555</t>
+        </is>
+      </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
           <t>3400930065556</t>
@@ -1711,7 +1835,11 @@
       <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>3030312</t>
+        </is>
+      </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
           <t>3400930303122</t>
@@ -1727,7 +1855,7 @@
         <v>366.23</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>351.98</v>
+        <v>352.02</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
@@ -1749,7 +1877,11 @@
       <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>3006578</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
           <t>3400930065785</t>
@@ -1787,7 +1919,11 @@
       <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>3625137</t>
+        </is>
+      </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
           <t>3400936251373</t>
@@ -1825,7 +1961,11 @@
       <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>3002858</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
           <t>3400930028582</t>
@@ -1841,7 +1981,7 @@
         <v>171.07</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>164.42</v>
+        <v>164.44</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
@@ -1863,7 +2003,11 @@
       <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>3778421</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
           <t>3400937784214</t>
@@ -1901,7 +2045,11 @@
       <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>6006071</t>
+        </is>
+      </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
@@ -1939,7 +2087,11 @@
       <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2673826</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
           <t>3400926738266</t>
@@ -1955,7 +2107,7 @@
         <v>7.62</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>7.32</v>
+        <v>7.33</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
@@ -1977,7 +2129,11 @@
       <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>3461546</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>3400934615467</t>
@@ -2015,7 +2171,11 @@
       <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2225720</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
           <t>3400922257204</t>
@@ -2053,7 +2213,11 @@
       <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>3006566</t>
+        </is>
+      </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
           <t>3400930065662</t>
@@ -2091,7 +2255,11 @@
       <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>3325406</t>
+        </is>
+      </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
           <t>3400933254063</t>
@@ -2129,7 +2297,11 @@
       <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>3006589</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
           <t>3400930065891</t>
@@ -2167,7 +2339,11 @@
       <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>9000008</t>
+        </is>
+      </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
@@ -2205,7 +2381,11 @@
       <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>3244079</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
           <t>3400932440795</t>
@@ -2243,7 +2423,11 @@
       <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>6223558</t>
+        </is>
+      </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
@@ -2281,7 +2465,11 @@
       <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>3029293</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
           <t>3400930292938</t>
@@ -2297,7 +2485,7 @@
         <v>313.27</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>301.08</v>
+        <v>301.11</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
@@ -2319,7 +2507,11 @@
       <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>3192750</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
           <t>3400931927501</t>
@@ -2357,7 +2549,11 @@
       <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>3535606</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
           <t>3400935356062</t>
@@ -2370,10 +2566,10 @@
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>4.51</v>
+        <v>4.43</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>4.51</v>
+        <v>4.43</v>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
@@ -2395,7 +2591,11 @@
       <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>3024437</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
           <t>3400930244371</t>
@@ -2411,7 +2611,7 @@
         <v>45.12</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>43.36</v>
+        <v>43.39</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
@@ -2433,7 +2633,11 @@
       <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>3293534</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
           <t>3400932935345</t>
@@ -2471,7 +2675,11 @@
       <c r="P52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>3464668</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
           <t>3400934646683</t>
@@ -2509,7 +2717,11 @@
       <c r="P53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>3066933</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
           <t>3400930669334</t>
@@ -2547,7 +2759,11 @@
       <c r="P54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>3687374</t>
+        </is>
+      </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
           <t>3400936873742</t>
@@ -2563,7 +2779,7 @@
         <v>19.92</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>19.15</v>
+        <v>19.17</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
@@ -2585,7 +2801,11 @@
       <c r="P55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>3820382</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
           <t>3400938203820</t>
@@ -2623,7 +2843,11 @@
       <c r="P56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>3351800</t>
+        </is>
+      </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
           <t>3400933518004</t>
@@ -2661,7 +2885,11 @@
       <c r="P57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2225393</t>
+        </is>
+      </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
           <t>3400922253930</t>
@@ -2677,7 +2905,7 @@
         <v>36.18</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>34.77</v>
+        <v>34.8</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
@@ -2699,7 +2927,11 @@
       <c r="P58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>3000376</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
           <t>3400930003763</t>
@@ -2715,7 +2947,7 @@
         <v>74.28</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>71.39</v>
+        <v>71.42</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
@@ -2737,7 +2969,11 @@
       <c r="P59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>3015110</t>
+        </is>
+      </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
           <t>3400930151105</t>
@@ -2753,7 +2989,7 @@
         <v>70.98999999999999</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>68.23</v>
+        <v>68.25</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
@@ -2775,7 +3011,11 @@
       <c r="P60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>3012140</t>
+        </is>
+      </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
           <t>3400930121405</t>
@@ -2813,7 +3053,11 @@
       <c r="P61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>3218969</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
           <t>3400932189694</t>
@@ -2851,7 +3095,11 @@
       <c r="P62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>3595583</t>
+        </is>
+      </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
           <t>3400935955838</t>
@@ -2889,7 +3137,11 @@
       <c r="P63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>3113638</t>
+        </is>
+      </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
           <t>3400931136385</t>
@@ -2927,7 +3179,11 @@
       <c r="P64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>3189363</t>
+        </is>
+      </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
           <t>3400931893639</t>
@@ -2965,7 +3221,11 @@
       <c r="P65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>3025862</t>
+        </is>
+      </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
           <t>3400930258620</t>
@@ -2981,7 +3241,7 @@
         <v>136.5</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>131.19</v>
+        <v>131.21</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
@@ -3003,7 +3263,11 @@
       <c r="P66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>3192253</t>
+        </is>
+      </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
           <t>3400931922537</t>
@@ -3041,7 +3305,11 @@
       <c r="P67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>3006568</t>
+        </is>
+      </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
           <t>3400930065686</t>
@@ -3079,7 +3347,11 @@
       <c r="P68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>3023000</t>
+        </is>
+      </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
           <t>3400930230008</t>
@@ -3117,7 +3389,11 @@
       <c r="P69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>3233153</t>
+        </is>
+      </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
           <t>3400932331536</t>
@@ -3155,7 +3431,11 @@
       <c r="P70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>3174284</t>
+        </is>
+      </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
           <t>3400931742845</t>
@@ -3193,7 +3473,11 @@
       <c r="P71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>6311785</t>
+        </is>
+      </c>
       <c r="B72" t="inlineStr"/>
       <c r="C72" s="2" t="inlineStr">
         <is>
@@ -3231,7 +3515,11 @@
       <c r="P72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>3006601</t>
+        </is>
+      </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
           <t>3400930066010</t>
@@ -3269,7 +3557,11 @@
       <c r="P73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>3707125</t>
+        </is>
+      </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
           <t>3400937071253</t>
@@ -3307,7 +3599,11 @@
       <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>3158575</t>
+        </is>
+      </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
           <t>3400931585756</t>
@@ -3345,7 +3641,11 @@
       <c r="P75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>3041867</t>
+        </is>
+      </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
           <t>3400930418673</t>
@@ -3361,7 +3661,7 @@
         <v>4.41</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>4.24</v>
+        <v>4.23</v>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
@@ -3383,7 +3683,11 @@
       <c r="P76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>4153396</t>
+        </is>
+      </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
           <t>3400941533969</t>
@@ -3421,7 +3725,11 @@
       <c r="P77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>3624698</t>
+        </is>
+      </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
           <t>3400936246980</t>
@@ -3459,7 +3767,11 @@
       <c r="P78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>3026454</t>
+        </is>
+      </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
           <t>3400930264546</t>
@@ -3497,7 +3809,11 @@
       <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>3025866</t>
+        </is>
+      </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
           <t>3400930258668</t>
@@ -3513,7 +3829,7 @@
         <v>181.48</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>174.42</v>
+        <v>174.45</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -3535,7 +3851,11 @@
       <c r="P80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>4168624</t>
+        </is>
+      </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
           <t>3400941686245</t>
@@ -3573,7 +3893,11 @@
       <c r="P81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>3025864</t>
+        </is>
+      </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
           <t>3400930258644</t>
@@ -3589,7 +3913,7 @@
         <v>136.5</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>131.19</v>
+        <v>131.21</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
@@ -3611,7 +3935,11 @@
       <c r="P82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>3513734</t>
+        </is>
+      </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
           <t>3400935137340</t>
@@ -3627,7 +3955,7 @@
         <v>11.84</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>11.38</v>
+        <v>11.4</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
@@ -3649,7 +3977,11 @@
       <c r="P83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>3391308</t>
+        </is>
+      </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
           <t>3400933913083</t>
@@ -3687,7 +4019,11 @@
       <c r="P84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr"/>
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>3747768</t>
+        </is>
+      </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
           <t>3400937477680</t>
@@ -3725,7 +4061,11 @@
       <c r="P85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>3279066</t>
+        </is>
+      </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
           <t>3400932790661</t>
@@ -3763,7 +4103,11 @@
       <c r="P86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr"/>
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>3021645</t>
+        </is>
+      </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
           <t>3400930216453</t>
@@ -3779,7 +4123,7 @@
         <v>74.28</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>71.39</v>
+        <v>71.42</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
@@ -3801,7 +4145,11 @@
       <c r="P87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>3029294</t>
+        </is>
+      </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
           <t>3400930292945</t>
@@ -3817,7 +4165,7 @@
         <v>313.27</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>301.08</v>
+        <v>301.11</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
@@ -3839,7 +4187,11 @@
       <c r="P88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>3135858</t>
+        </is>
+      </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
           <t>3400931358589</t>
@@ -3877,7 +4229,11 @@
       <c r="P89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>3264550</t>
+        </is>
+      </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
           <t>3400932645503</t>
@@ -3915,7 +4271,11 @@
       <c r="P90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>3023497</t>
+        </is>
+      </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
           <t>3400930234976</t>
@@ -3953,7 +4313,11 @@
       <c r="P91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>3499945</t>
+        </is>
+      </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
           <t>3400934999451</t>
@@ -3991,7 +4355,11 @@
       <c r="P92" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr"/>
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>3105283</t>
+        </is>
+      </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
           <t>3400931052838</t>
@@ -4029,7 +4397,11 @@
       <c r="P93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>3118794</t>
+        </is>
+      </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
           <t>3400931187943</t>
@@ -4067,7 +4439,11 @@
       <c r="P94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr"/>
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>3006557</t>
+        </is>
+      </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
           <t>3400930065570</t>
@@ -4105,7 +4481,11 @@
       <c r="P95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>3228577</t>
+        </is>
+      </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
           <t>3400932285778</t>
@@ -4121,7 +4501,7 @@
         <v>6.98</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>6.71</v>
+        <v>6.98</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr"/>
@@ -4143,7 +4523,11 @@
       <c r="P96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>4066912</t>
+        </is>
+      </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" s="2" t="inlineStr">
         <is>
@@ -4181,7 +4565,11 @@
       <c r="P97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr"/>
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>3008456</t>
+        </is>
+      </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
           <t>3400930084564</t>
@@ -4219,7 +4607,11 @@
       <c r="P98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2217904</t>
+        </is>
+      </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
           <t>3400922179049</t>
@@ -4257,7 +4649,11 @@
       <c r="P99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>3020488</t>
+        </is>
+      </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
           <t>3400930204887</t>
@@ -4295,7 +4691,11 @@
       <c r="P100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr"/>
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>3021648</t>
+        </is>
+      </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
           <t>3400930216484</t>
@@ -4311,7 +4711,7 @@
         <v>74.28</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>71.39</v>
+        <v>71.42</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr"/>
@@ -4333,7 +4733,11 @@
       <c r="P101" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>3570614</t>
+        </is>
+      </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
           <t>3400935706140</t>
@@ -4371,7 +4775,11 @@
       <c r="P102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>3026024</t>
+        </is>
+      </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
           <t>3400930260241</t>
@@ -4387,7 +4795,7 @@
         <v>157.37</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>151.25</v>
+        <v>151.27</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
@@ -4409,7 +4817,11 @@
       <c r="P103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>3529422</t>
+        </is>
+      </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
           <t>3400935294227</t>
@@ -4447,7 +4859,11 @@
       <c r="P104" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>3189819</t>
+        </is>
+      </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
           <t>3400931898191</t>
@@ -4485,7 +4901,11 @@
       <c r="P105" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr"/>
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>3192767</t>
+        </is>
+      </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
           <t>3400931927679</t>
@@ -4523,7 +4943,11 @@
       <c r="P106" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr"/>
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>3348413</t>
+        </is>
+      </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
           <t>3400933484132</t>
@@ -4561,7 +4985,11 @@
       <c r="P107" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>3422397</t>
+        </is>
+      </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
           <t>3400934223976</t>
@@ -4599,7 +5027,11 @@
       <c r="P108" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2735007</t>
+        </is>
+      </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
           <t>3400927350078</t>
@@ -4615,7 +5047,7 @@
         <v>30.09</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>28.92</v>
+        <v>28.94</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
@@ -4637,7 +5069,11 @@
       <c r="P109" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr"/>
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>3480940</t>
+        </is>
+      </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
           <t>3400934809408</t>
@@ -4675,7 +5111,11 @@
       <c r="P110" t="inlineStr"/>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr"/>
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>3230829</t>
+        </is>
+      </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
           <t>3400932308293</t>
@@ -4713,7 +5153,11 @@
       <c r="P111" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr"/>
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>3446417</t>
+        </is>
+      </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
           <t>3400934464171</t>
@@ -4751,7 +5195,11 @@
       <c r="P112" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>3644146</t>
+        </is>
+      </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
           <t>3400936441460</t>
@@ -4789,7 +5237,11 @@
       <c r="P113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr"/>
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>3153342</t>
+        </is>
+      </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
           <t>3400931533429</t>
@@ -4827,7 +5279,11 @@
       <c r="P114" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2669210</t>
+        </is>
+      </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
           <t>3400926692100</t>
@@ -4865,7 +5321,11 @@
       <c r="P115" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>3412594</t>
+        </is>
+      </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
           <t>3400934125942</t>
@@ -4903,7 +5363,11 @@
       <c r="P116" t="inlineStr"/>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>3001667</t>
+        </is>
+      </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
           <t>3400930016671</t>
@@ -4919,7 +5383,7 @@
         <v>32.31</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>31.05</v>
+        <v>31.08</v>
       </c>
       <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr"/>
@@ -4941,7 +5405,11 @@
       <c r="P117" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>5437210</t>
+        </is>
+      </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" s="2" t="inlineStr">
         <is>
@@ -4979,7 +5447,11 @@
       <c r="P118" t="inlineStr"/>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>3105308</t>
+        </is>
+      </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
           <t>3400931053088</t>
@@ -5017,7 +5489,11 @@
       <c r="P119" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>3140500</t>
+        </is>
+      </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
           <t>3400931405009</t>
@@ -5055,7 +5531,11 @@
       <c r="P120" t="inlineStr"/>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2788676</t>
+        </is>
+      </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
           <t>3400927886768</t>
@@ -5093,7 +5573,11 @@
       <c r="P121" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>3419538</t>
+        </is>
+      </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
           <t>3400934195389</t>
@@ -5131,7 +5615,11 @@
       <c r="P122" t="inlineStr"/>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>3019529</t>
+        </is>
+      </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
           <t>3400930195291</t>
@@ -5169,7 +5657,11 @@
       <c r="P123" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>3403589</t>
+        </is>
+      </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
           <t>3400934035890</t>
@@ -5207,7 +5699,11 @@
       <c r="P124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2678410</t>
+        </is>
+      </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
           <t>3400926784102</t>
@@ -5245,7 +5741,11 @@
       <c r="P125" t="inlineStr"/>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>3023498</t>
+        </is>
+      </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
           <t>3400930234983</t>
@@ -5283,7 +5783,11 @@
       <c r="P126" t="inlineStr"/>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>3026231</t>
+        </is>
+      </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
           <t>3400930262313</t>
@@ -5321,7 +5825,11 @@
       <c r="P127" t="inlineStr"/>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>3005328</t>
+        </is>
+      </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
           <t>3400930053287</t>
@@ -5359,7 +5867,11 @@
       <c r="P128" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>3491240</t>
+        </is>
+      </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
           <t>3400934912405</t>
@@ -5397,7 +5909,11 @@
       <c r="P129" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>3012142</t>
+        </is>
+      </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
           <t>3400930121429</t>
@@ -5413,7 +5929,7 @@
         <v>4.72</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>4.54</v>
+        <v>4.53</v>
       </c>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr"/>
@@ -5435,7 +5951,11 @@
       <c r="P130" t="inlineStr"/>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>3338461</t>
+        </is>
+      </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
           <t>3400933384616</t>
@@ -5473,7 +5993,11 @@
       <c r="P131" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr"/>
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>3015793</t>
+        </is>
+      </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
           <t>3400930157930</t>
@@ -5511,7 +6035,11 @@
       <c r="P132" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr"/>
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>3219294</t>
+        </is>
+      </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
           <t>3400932192946</t>
@@ -5549,7 +6077,11 @@
       <c r="P133" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr"/>
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>3232018</t>
+        </is>
+      </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
           <t>3400932320189</t>
@@ -5587,7 +6119,11 @@
       <c r="P134" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr"/>
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>3003791</t>
+        </is>
+      </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
           <t>3400930037911</t>
@@ -5625,7 +6161,11 @@
       <c r="P135" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr"/>
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>3442307</t>
+        </is>
+      </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
           <t>3400934423079</t>
@@ -5663,7 +6203,11 @@
       <c r="P136" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr"/>
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>3162329</t>
+        </is>
+      </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
           <t>3400931623298</t>
@@ -5701,7 +6245,11 @@
       <c r="P137" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr"/>
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>3003790</t>
+        </is>
+      </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
           <t>3400930037904</t>
@@ -5777,7 +6325,11 @@
       <c r="P139" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr"/>
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2685798</t>
+        </is>
+      </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
           <t>3400926857981</t>
@@ -5793,7 +6345,7 @@
         <v>51.83</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>49.81</v>
+        <v>49.84</v>
       </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
@@ -5815,7 +6367,11 @@
       <c r="P140" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr"/>
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>3024785</t>
+        </is>
+      </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
           <t>3400930247853</t>
@@ -5831,7 +6387,7 @@
         <v>52.31</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>50.28</v>
+        <v>50.3</v>
       </c>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
@@ -5853,7 +6409,11 @@
       <c r="P141" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr"/>
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>3677387</t>
+        </is>
+      </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
           <t>3400936773875</t>
@@ -5869,7 +6429,7 @@
         <v>19.92</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>19.15</v>
+        <v>19.17</v>
       </c>
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
@@ -5891,7 +6451,11 @@
       <c r="P142" t="inlineStr"/>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr"/>
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>3772298</t>
+        </is>
+      </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
           <t>3400937722988</t>
@@ -5907,7 +6471,7 @@
         <v>33.59</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>32.28</v>
+        <v>32.31</v>
       </c>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
@@ -5929,7 +6493,11 @@
       <c r="P143" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr"/>
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>3450778</t>
+        </is>
+      </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
           <t>3400934507786</t>
@@ -5967,7 +6535,11 @@
       <c r="P144" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr"/>
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>3015849</t>
+        </is>
+      </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
           <t>3400930158494</t>
@@ -6005,7 +6577,11 @@
       <c r="P145" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr"/>
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>3295510</t>
+        </is>
+      </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
           <t>3400932955107</t>
@@ -6043,7 +6619,11 @@
       <c r="P146" t="inlineStr"/>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr"/>
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>3480986</t>
+        </is>
+      </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
           <t>3400934809866</t>
@@ -6081,7 +6661,11 @@
       <c r="P147" t="inlineStr"/>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr"/>
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>3003792</t>
+        </is>
+      </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
           <t>3400930037928</t>
@@ -6119,7 +6703,11 @@
       <c r="P148" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr"/>
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>3031116</t>
+        </is>
+      </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
           <t>3400930311165</t>
@@ -6157,7 +6745,11 @@
       <c r="P149" t="inlineStr"/>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr"/>
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>7800001</t>
+        </is>
+      </c>
       <c r="B150" t="inlineStr"/>
       <c r="C150" s="2" t="inlineStr">
         <is>
@@ -6195,7 +6787,11 @@
       <c r="P150" t="inlineStr"/>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr"/>
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>3057302</t>
+        </is>
+      </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
           <t>3400930573020</t>
@@ -6233,7 +6829,11 @@
       <c r="P151" t="inlineStr"/>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr"/>
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>3006618</t>
+        </is>
+      </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
           <t>3400930066188</t>
@@ -6271,7 +6871,11 @@
       <c r="P152" t="inlineStr"/>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr"/>
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>3207026</t>
+        </is>
+      </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
           <t>3400932070268</t>
@@ -6309,7 +6913,11 @@
       <c r="P153" t="inlineStr"/>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr"/>
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>3015804</t>
+        </is>
+      </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
           <t>3400930158043</t>
@@ -6347,7 +6955,11 @@
       <c r="P154" t="inlineStr"/>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr"/>
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>3641662</t>
+        </is>
+      </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
           <t>3400936416628</t>
@@ -6385,7 +6997,11 @@
       <c r="P155" t="inlineStr"/>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr"/>
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>3768902</t>
+        </is>
+      </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
           <t>3400937689021</t>
@@ -6423,7 +7039,11 @@
       <c r="P156" t="inlineStr"/>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr"/>
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>3039698</t>
+        </is>
+      </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
           <t>3400930396988</t>
@@ -6461,7 +7081,11 @@
       <c r="P157" t="inlineStr"/>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr"/>
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>3027121</t>
+        </is>
+      </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
           <t>3400930271216</t>
@@ -6499,7 +7123,11 @@
       <c r="P158" t="inlineStr"/>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr"/>
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>3025251</t>
+        </is>
+      </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
           <t>3400930252512</t>
@@ -6537,7 +7165,11 @@
       <c r="P159" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr"/>
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>3113644</t>
+        </is>
+      </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
           <t>3400931136446</t>
@@ -6575,7 +7207,11 @@
       <c r="P160" t="inlineStr"/>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr"/>
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2761996</t>
+        </is>
+      </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
           <t>3400927619960</t>
@@ -6613,7 +7249,11 @@
       <c r="P161" t="inlineStr"/>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr"/>
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>3010861</t>
+        </is>
+      </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
           <t>3400930108611</t>
@@ -6651,7 +7291,11 @@
       <c r="P162" t="inlineStr"/>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr"/>
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>3480911</t>
+        </is>
+      </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
           <t>3400934809118</t>
@@ -6689,7 +7333,11 @@
       <c r="P163" t="inlineStr"/>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr"/>
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>3014595</t>
+        </is>
+      </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
           <t>3400930145951</t>
@@ -6727,7 +7375,11 @@
       <c r="P164" t="inlineStr"/>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr"/>
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>3204654</t>
+        </is>
+      </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
           <t>3400932046546</t>
@@ -6765,7 +7417,11 @@
       <c r="P165" t="inlineStr"/>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr"/>
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>3024059</t>
+        </is>
+      </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
           <t>3400930240595</t>
@@ -6781,7 +7437,7 @@
         <v>9.35</v>
       </c>
       <c r="F166" s="3" t="n">
-        <v>8.99</v>
+        <v>8.98</v>
       </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="inlineStr"/>
@@ -6803,7 +7459,11 @@
       <c r="P166" t="inlineStr"/>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr"/>
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>3339756</t>
+        </is>
+      </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
           <t>3400933397562</t>
@@ -6841,7 +7501,11 @@
       <c r="P167" t="inlineStr"/>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr"/>
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>3027120</t>
+        </is>
+      </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
           <t>3400930271209</t>
@@ -6879,7 +7543,11 @@
       <c r="P168" t="inlineStr"/>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr"/>
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>4925031</t>
+        </is>
+      </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
           <t>3400949250318</t>
@@ -6895,7 +7563,7 @@
         <v>4.42</v>
       </c>
       <c r="F169" s="3" t="n">
-        <v>4.25</v>
+        <v>4.24</v>
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr"/>
@@ -6917,7 +7585,11 @@
       <c r="P169" t="inlineStr"/>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr"/>
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>3025863</t>
+        </is>
+      </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
           <t>3400930258637</t>
@@ -6933,7 +7605,7 @@
         <v>136.5</v>
       </c>
       <c r="F170" s="3" t="n">
-        <v>131.19</v>
+        <v>131.21</v>
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr"/>
@@ -6955,7 +7627,11 @@
       <c r="P170" t="inlineStr"/>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr"/>
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>4194567</t>
+        </is>
+      </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
           <t>3400941945670</t>
@@ -6993,7 +7669,11 @@
       <c r="P171" t="inlineStr"/>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr"/>
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>3007978</t>
+        </is>
+      </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
           <t>3400930079782</t>
@@ -7009,7 +7689,7 @@
         <v>29.5</v>
       </c>
       <c r="F172" s="3" t="n">
-        <v>28.35</v>
+        <v>28.38</v>
       </c>
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr"/>
@@ -7031,7 +7711,11 @@
       <c r="P172" t="inlineStr"/>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr"/>
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>3149978</t>
+        </is>
+      </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
           <t>3400931499787</t>
@@ -7069,7 +7753,11 @@
       <c r="P173" t="inlineStr"/>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr"/>
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>3002411</t>
+        </is>
+      </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
           <t>3400930024119</t>
@@ -7107,7 +7795,11 @@
       <c r="P174" t="inlineStr"/>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr"/>
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2675268</t>
+        </is>
+      </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
           <t>3400926752682</t>
@@ -7145,7 +7837,11 @@
       <c r="P175" t="inlineStr"/>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr"/>
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>3065253</t>
+        </is>
+      </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
           <t>3400930652534</t>
@@ -7183,7 +7879,11 @@
       <c r="P176" t="inlineStr"/>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr"/>
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>3588755</t>
+        </is>
+      </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
           <t>3400935887559</t>
@@ -7221,7 +7921,11 @@
       <c r="P177" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr"/>
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>3031324</t>
+        </is>
+      </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
           <t>3400930313244</t>
@@ -7259,7 +7963,11 @@
       <c r="P178" t="inlineStr"/>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr"/>
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>3004007</t>
+        </is>
+      </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
           <t>3400930040072</t>
@@ -7275,7 +7983,7 @@
         <v>31.19</v>
       </c>
       <c r="F179" s="3" t="n">
-        <v>29.98</v>
+        <v>30</v>
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr"/>
@@ -7297,7 +8005,11 @@
       <c r="P179" t="inlineStr"/>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr"/>
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>3516690</t>
+        </is>
+      </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
           <t>3400935166906</t>
@@ -7313,7 +8025,7 @@
         <v>14.5</v>
       </c>
       <c r="F180" s="3" t="n">
-        <v>13.94</v>
+        <v>13.96</v>
       </c>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr"/>
@@ -7335,7 +8047,11 @@
       <c r="P180" t="inlineStr"/>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr"/>
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>3263711</t>
+        </is>
+      </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
           <t>3400932637119</t>
@@ -7373,7 +8089,11 @@
       <c r="P181" t="inlineStr"/>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr"/>
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>3032215</t>
+        </is>
+      </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
           <t>3400930322154</t>
@@ -7389,7 +8109,7 @@
         <v>70.98999999999999</v>
       </c>
       <c r="F182" s="3" t="n">
-        <v>68.23</v>
+        <v>68.25</v>
       </c>
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr"/>
@@ -7411,7 +8131,11 @@
       <c r="P182" t="inlineStr"/>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr"/>
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>3248781</t>
+        </is>
+      </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
           <t>3400932487813</t>
@@ -7449,7 +8173,11 @@
       <c r="P183" t="inlineStr"/>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr"/>
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>3442997</t>
+        </is>
+      </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
           <t>3400934429972</t>
@@ -7487,7 +8215,11 @@
       <c r="P184" t="inlineStr"/>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr"/>
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>3301802</t>
+        </is>
+      </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
           <t>3400933018023</t>
@@ -7525,7 +8257,11 @@
       <c r="P185" t="inlineStr"/>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr"/>
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>3274850</t>
+        </is>
+      </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
           <t>3400932748501</t>
@@ -7563,7 +8299,11 @@
       <c r="P186" t="inlineStr"/>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr"/>
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>3649793</t>
+        </is>
+      </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
           <t>3400936497931</t>
@@ -7601,7 +8341,11 @@
       <c r="P187" t="inlineStr"/>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr"/>
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>3063219</t>
+        </is>
+      </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
           <t>3400930632192</t>
@@ -7639,7 +8383,11 @@
       <c r="P188" t="inlineStr"/>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr"/>
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>3707102</t>
+        </is>
+      </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
           <t>3400937071024</t>
@@ -7715,7 +8463,11 @@
       <c r="P190" t="inlineStr"/>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr"/>
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>3285552</t>
+        </is>
+      </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
           <t>3400932855520</t>
@@ -7753,7 +8505,11 @@
       <c r="P191" t="inlineStr"/>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr"/>
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>3278173</t>
+        </is>
+      </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
           <t>3400932781737</t>
@@ -7791,7 +8547,11 @@
       <c r="P192" t="inlineStr"/>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr"/>
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>3636684</t>
+        </is>
+      </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
           <t>3400936366848</t>
@@ -7829,7 +8589,11 @@
       <c r="P193" t="inlineStr"/>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr"/>
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>3239948</t>
+        </is>
+      </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
           <t>3400932399482</t>
@@ -7867,7 +8631,11 @@
       <c r="P194" t="inlineStr"/>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr"/>
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>3481017</t>
+        </is>
+      </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
           <t>3400934810176</t>
@@ -7905,7 +8673,11 @@
       <c r="P195" t="inlineStr"/>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr"/>
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>6025385</t>
+        </is>
+      </c>
       <c r="B196" t="inlineStr"/>
       <c r="C196" s="2" t="inlineStr">
         <is>
@@ -7943,7 +8715,11 @@
       <c r="P196" t="inlineStr"/>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr"/>
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>3222379</t>
+        </is>
+      </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
           <t>3400932223794</t>
@@ -7981,7 +8757,11 @@
       <c r="P197" t="inlineStr"/>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr"/>
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>3413613</t>
+        </is>
+      </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
           <t>3400934136139</t>
@@ -8019,7 +8799,11 @@
       <c r="P198" t="inlineStr"/>
     </row>
     <row r="199">
-      <c r="A199" t="inlineStr"/>
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>3691849</t>
+        </is>
+      </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
           <t>3400936918498</t>
@@ -8057,7 +8841,11 @@
       <c r="P199" t="inlineStr"/>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr"/>
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2795647</t>
+        </is>
+      </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
           <t>3400927956478</t>
@@ -8095,7 +8883,11 @@
       <c r="P200" t="inlineStr"/>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr"/>
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>3012144</t>
+        </is>
+      </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
           <t>3400930121443</t>

</xml_diff>